<commit_message>
Minor fixes and improvements
</commit_message>
<xml_diff>
--- a/Statistik för användarupplevelseprojekt (UX-projekt).xlsx
+++ b/Statistik för användarupplevelseprojekt (UX-projekt).xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joakim.Hasselblad\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://paab159-my.sharepoint.com/personal/joakim_hasselblad_pm3_se1/Documents/Omvärldsbevakning/Statistik/Simple_Stats_for_UX_Projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F89A4F4C-7DED-4DBD-867F-34F907D8BD62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="8_{F89A4F4C-7DED-4DBD-867F-34F907D8BD62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77471F99-2CE2-4893-91BB-893FF055E078}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="123">
   <si>
     <t>Syntax:</t>
   </si>
@@ -391,36 +391,9 @@
     <t>Vidd</t>
   </si>
   <si>
-    <t>efter att omfången konverterats till rangordningar!</t>
-  </si>
-  <si>
     <t>Pearsons r - samband i kvantitativa data</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">T-test </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>P</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> = </t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">Chi kvadrat (Chi Square) </t>
   </si>
   <si>
@@ -436,13 +409,7 @@
     <t>Lutning</t>
   </si>
   <si>
-    <t>Att beräkna skärningspunkt och lutning för korrelerad data</t>
-  </si>
-  <si>
     <t>Samband</t>
-  </si>
-  <si>
-    <t>Samband - att visa korrelationer</t>
   </si>
   <si>
     <t>Testar om skillnader i kvalitativa data är statistiskt signifikanta</t>
@@ -490,30 +457,6 @@
   </si>
   <si>
     <t xml:space="preserve">T-test p = </t>
-  </si>
-  <si>
-    <r>
-      <t>Chi Square p</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>=</t>
-    </r>
   </si>
   <si>
     <r>
@@ -568,9 +511,6 @@
   </si>
   <si>
     <t>Översikt Statistik för användarupplevelseprojekt</t>
-  </si>
-  <si>
-    <t>Att bekriva variationen i en datamängd</t>
   </si>
   <si>
     <t>Jämförelse skillnader - att visa konfidensintervall</t>
@@ -654,15 +594,9 @@
     </r>
   </si>
   <si>
-    <t>Test av samband mellan kvalitativa variabler (eller ej normalfördelade kvantitativa variabler)</t>
-  </si>
-  <si>
     <t>Jämföra skillnader</t>
   </si>
   <si>
-    <t>Om intervallen inte överlappar är skillnaden statistiskt signifikant vid den valda konfidensnivån, dvs. vi kan anta att det faktiskt finns en skillnad i den större populationen</t>
-  </si>
-  <si>
     <t>Mäter styrkan och riktningen hos ett linjärt samband mellan två kvantitativa variabler</t>
   </si>
   <si>
@@ -730,6 +664,56 @@
   </si>
   <si>
     <t>i kvadrat</t>
+  </si>
+  <si>
+    <t>Att bekriva variationen i en variabel</t>
+  </si>
+  <si>
+    <t>Rangkorrelation; test av samband mellan kvalitativa variabler (eller ej normalfördelade kvantitativa variabler)</t>
+  </si>
+  <si>
+    <t>=RANG:MED(tal;referens;[ordning])</t>
+  </si>
+  <si>
+    <t>=KORREL() används efter att omfången konverterats till rangordningar med =RANG.MED(), se kolumnerna E och F</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <r>
+      <t>Chi Square p</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>=</t>
+    </r>
+  </si>
+  <si>
+    <t>Om intervallen inte överlappar är skillnaden statistiskt signifikant vid den valda konfidensnivån, dvs. vi kan anta att det faktiskt finns en skillnad i den större populationen. Jfr t-test p.</t>
+  </si>
+  <si>
+    <t>Att beräkna skärningspunkt och lutning för korrelerad data (trendlinje)</t>
+  </si>
+  <si>
+    <t>Samband - att visa korrelation</t>
   </si>
 </sst>
 </file>
@@ -743,7 +727,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -882,6 +866,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -911,7 +903,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -989,7 +981,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1043,6 +1034,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlänk" xfId="1" builtinId="8"/>
@@ -2613,7 +2608,7 @@
                 <a:sysClr val="windowText" lastClr="000000"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>"I vårt urval hade användare med premiumkonton i genomsnitt drygt 10 personer fler i sina nätverk än användare med gratiskonton</a:t>
+            <a:t>"I vår undersökningsgrupp hade användare med premiumkonton i genomsnitt drygt 10 personer fler i sina nätverk än användare med gratiskonton</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="sv-SE" sz="1050" i="1" baseline="0">
@@ -2657,6 +2652,156 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>120650</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>44450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>260350</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="textruta 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3EE3380-5192-A92E-D40B-3DCB084A780C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5372100" y="1041400"/>
+          <a:ext cx="2635250" cy="692150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFF00"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1000"/>
+            <a:t>Skalan går mellan -1 och 1, där 0 indikerar att inget samband finns mellan variablerna. Det aktuella värdet visar alltså på ett starkt negativt samband mellan variablerna.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>70554</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>423334</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>134055</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>134762</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="textruta 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04975F7F-B47F-45C7-9437-4110B5012501}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8748887" y="1594556"/>
+          <a:ext cx="2730501" cy="692150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFF00"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1000"/>
+            <a:t>Skalan går mellan -1 och 1, där 0 indikerar att inget samband finns mellan variablerna. Det aktuella värdet visar alltså på ett ganska starkt negativt samband mellan variablerna.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
@@ -2691,7 +2836,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -2973,15 +3118,15 @@
   <sheetData>
     <row r="1" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="26" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="56" t="s">
-        <v>79</v>
-      </c>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
+      <c r="A2" s="55" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
@@ -2998,12 +3143,12 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="36" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -3023,62 +3168,62 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="36" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="36" t="s">
-        <v>75</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="13" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="12"/>
     </row>
     <row r="16" spans="1:11" ht="13" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="55" t="s">
+      <c r="A16" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="55"/>
-      <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
-      <c r="E16" s="55"/>
-      <c r="F16" s="55"/>
-      <c r="G16" s="55"/>
-      <c r="H16" s="55"/>
-      <c r="I16" s="55"/>
-      <c r="J16" s="55"/>
-      <c r="K16" s="55"/>
+      <c r="B16" s="54"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="54"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="54"/>
+      <c r="G16" s="54"/>
+      <c r="H16" s="54"/>
+      <c r="I16" s="54"/>
+      <c r="J16" s="54"/>
+      <c r="K16" s="54"/>
     </row>
     <row r="17" spans="1:11" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="55"/>
-      <c r="B17" s="55"/>
-      <c r="C17" s="55"/>
-      <c r="D17" s="55"/>
-      <c r="E17" s="55"/>
-      <c r="F17" s="55"/>
-      <c r="G17" s="55"/>
-      <c r="H17" s="55"/>
-      <c r="I17" s="55"/>
-      <c r="J17" s="55"/>
-      <c r="K17" s="55"/>
+      <c r="A17" s="54"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54"/>
+      <c r="G17" s="54"/>
+      <c r="H17" s="54"/>
+      <c r="I17" s="54"/>
+      <c r="J17" s="54"/>
+      <c r="K17" s="54"/>
     </row>
     <row r="18" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="55"/>
-      <c r="B18" s="55"/>
-      <c r="C18" s="55"/>
-      <c r="D18" s="55"/>
-      <c r="E18" s="55"/>
-      <c r="F18" s="55"/>
-      <c r="G18" s="55"/>
-      <c r="H18" s="55"/>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="55"/>
+      <c r="A18" s="54"/>
+      <c r="B18" s="54"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="54"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="54"/>
+      <c r="J18" s="54"/>
+      <c r="K18" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3120,12 +3265,12 @@
   <sheetData>
     <row r="1" spans="1:25" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>73</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="13" x14ac:dyDescent="0.3">
@@ -3133,12 +3278,12 @@
         <v>0</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:25" ht="13" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
@@ -3302,7 +3447,7 @@
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F12" s="11">
         <f>INTERCEPT(C9:C24,B9:B24)</f>
@@ -3336,7 +3481,7 @@
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="11" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F13" s="11">
         <f>SLOPE(C9:C24,B9:B24)</f>
@@ -3920,17 +4065,17 @@
         <v>0</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B5" s="9" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B6" s="9" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:23" s="12" customFormat="1" x14ac:dyDescent="0.3">
@@ -4021,8 +4166,8 @@
         <v>30</v>
       </c>
       <c r="F11" s="11"/>
-      <c r="G11" s="42" t="s">
-        <v>100</v>
+      <c r="G11" s="41" t="s">
+        <v>92</v>
       </c>
       <c r="H11" s="25" t="s">
         <v>7</v>
@@ -4138,8 +4283,8 @@
         <v>1</v>
       </c>
       <c r="J14" s="11"/>
-      <c r="K14" s="53" t="s">
-        <v>116</v>
+      <c r="K14" s="52" t="s">
+        <v>108</v>
       </c>
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
@@ -4169,8 +4314,8 @@
         <v>55</v>
       </c>
       <c r="F15" s="11"/>
-      <c r="G15" s="42" t="s">
-        <v>101</v>
+      <c r="G15" s="41" t="s">
+        <v>93</v>
       </c>
       <c r="H15" s="25">
         <v>2</v>
@@ -4390,7 +4535,7 @@
       <c r="G21" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H21" s="52"/>
+      <c r="H21" s="51"/>
       <c r="J21" s="11"/>
       <c r="K21" s="11"/>
       <c r="L21" s="11"/>
@@ -4506,7 +4651,7 @@
         <v>42</v>
       </c>
       <c r="J24" s="11"/>
-      <c r="K24" s="54"/>
+      <c r="K24" s="53"/>
       <c r="L24" s="11"/>
       <c r="M24" s="11"/>
       <c r="N24" s="11"/>
@@ -4753,8 +4898,8 @@
         <v>50000</v>
       </c>
       <c r="F13" s="11"/>
-      <c r="G13" s="42" t="s">
-        <v>80</v>
+      <c r="G13" s="41" t="s">
+        <v>76</v>
       </c>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
@@ -5049,7 +5194,7 @@
     </row>
     <row r="2" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
       <c r="H2" s="23"/>
       <c r="J2" s="23"/>
@@ -5063,7 +5208,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>52</v>
@@ -5073,7 +5218,7 @@
     </row>
     <row r="5" spans="1:25" s="12" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>53</v>
@@ -5083,7 +5228,7 @@
     </row>
     <row r="6" spans="1:25" s="12" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>54</v>
@@ -5093,7 +5238,7 @@
     </row>
     <row r="7" spans="1:25" s="12" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="B7" s="19" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>55</v>
@@ -5138,10 +5283,10 @@
         <v>12</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="D10" s="27" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="E10" s="20"/>
       <c r="F10" s="11"/>
@@ -5188,7 +5333,7 @@
         <v>20</v>
       </c>
       <c r="I11" s="11"/>
-      <c r="J11" s="43"/>
+      <c r="J11" s="42"/>
       <c r="K11" s="11"/>
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
@@ -5861,6 +6006,8 @@
     <col min="2" max="2" width="15.1796875" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="7" customWidth="1"/>
+    <col min="7" max="7" width="4" customWidth="1"/>
+    <col min="8" max="9" width="10.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="15.5" x14ac:dyDescent="0.35">
@@ -5870,7 +6017,7 @@
     </row>
     <row r="2" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -5879,7 +6026,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -5961,7 +6108,7 @@
         <v>-0.80447131470781463</v>
       </c>
       <c r="G9" s="11"/>
-      <c r="H9" s="29"/>
+      <c r="H9" s="60"/>
       <c r="I9" s="11"/>
       <c r="J9" s="11"/>
       <c r="K9" s="11"/>
@@ -6075,15 +6222,15 @@
         <v>28</v>
       </c>
       <c r="D13" s="11"/>
-      <c r="E13" s="57" t="s">
-        <v>82</v>
-      </c>
-      <c r="F13" s="58"/>
-      <c r="G13" s="58"/>
-      <c r="H13" s="58"/>
-      <c r="I13" s="58"/>
-      <c r="J13" s="58"/>
-      <c r="K13" s="58"/>
+      <c r="E13" s="56" t="s">
+        <v>78</v>
+      </c>
+      <c r="F13" s="57"/>
+      <c r="G13" s="57"/>
+      <c r="H13" s="57"/>
+      <c r="I13" s="57"/>
+      <c r="J13" s="57"/>
+      <c r="K13" s="57"/>
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
       <c r="N13" s="11"/>
@@ -6107,13 +6254,13 @@
         <v>21</v>
       </c>
       <c r="D14" s="11"/>
-      <c r="E14" s="58"/>
-      <c r="F14" s="58"/>
-      <c r="G14" s="58"/>
-      <c r="H14" s="58"/>
-      <c r="I14" s="58"/>
-      <c r="J14" s="58"/>
-      <c r="K14" s="58"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="57"/>
+      <c r="I14" s="57"/>
+      <c r="J14" s="57"/>
+      <c r="K14" s="57"/>
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
       <c r="N14" s="11"/>
@@ -6137,13 +6284,13 @@
         <v>4</v>
       </c>
       <c r="D15" s="11"/>
-      <c r="E15" s="58"/>
-      <c r="F15" s="58"/>
-      <c r="G15" s="58"/>
-      <c r="H15" s="58"/>
-      <c r="I15" s="58"/>
-      <c r="J15" s="58"/>
-      <c r="K15" s="58"/>
+      <c r="E15" s="57"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="57"/>
+      <c r="I15" s="57"/>
+      <c r="J15" s="57"/>
+      <c r="K15" s="57"/>
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
       <c r="N15" s="11"/>
@@ -6278,7 +6425,7 @@
       </c>
       <c r="D20" s="11"/>
       <c r="E20" s="31" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F20" s="29">
         <f>TDIST(F19,SUM(C8:C23-2),2)</f>
@@ -6606,6 +6753,7 @@
     <mergeCell ref="E13:K15"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6614,7 +6762,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.453125" style="12"/>
@@ -6632,63 +6780,45 @@
   <sheetData>
     <row r="1" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="34" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>111</v>
+      <c r="B4" s="9" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="13" x14ac:dyDescent="0.3">
-      <c r="B5" s="37" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" ht="39" x14ac:dyDescent="0.3">
-      <c r="B7" s="35" t="s">
+      <c r="B5" s="19" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="13" x14ac:dyDescent="0.3">
+      <c r="B6" s="61" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="39" x14ac:dyDescent="0.3">
+      <c r="B8" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35" t="s">
+      <c r="C8" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="35" t="s">
+      <c r="F8" s="35" t="s">
         <v>20</v>
-      </c>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B8" s="11">
-        <v>5.2</v>
-      </c>
-      <c r="C8" s="11">
-        <v>4</v>
-      </c>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11">
-        <f t="shared" ref="E8:F8" si="0">_xlfn.RANK.AVG(B8,B$8:B$23,1)</f>
-        <v>11</v>
-      </c>
-      <c r="F8" s="11">
-        <f t="shared" si="0"/>
-        <v>14</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="11"/>
@@ -6697,269 +6827,262 @@
       <c r="K8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="1:14" ht="13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B9" s="11">
-        <v>3.4</v>
+        <v>5.2</v>
       </c>
       <c r="C9" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="11">
-        <f t="shared" ref="E9:F9" si="1">_xlfn.RANK.AVG(B9,B$8:B$23,1)</f>
-        <v>5.5</v>
+        <f t="shared" ref="E9:F9" si="0">_xlfn.RANK.AVG(B9,B$9:B$24,1)</f>
+        <v>11</v>
       </c>
       <c r="F9" s="11">
-        <f t="shared" si="1"/>
-        <v>9</v>
+        <f t="shared" si="0"/>
+        <v>14</v>
       </c>
       <c r="G9" s="11"/>
-      <c r="H9" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="I9" s="29">
-        <f>CORREL(E8:E23,F8:F23)</f>
-        <v>-0.74588967113847993</v>
-      </c>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
       <c r="J9" s="11"/>
       <c r="K9" s="11"/>
       <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="B10" s="11">
-        <v>6.1</v>
+        <v>3.4</v>
       </c>
       <c r="C10" s="11">
         <v>3</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="11">
-        <f t="shared" ref="E10:F10" si="2">_xlfn.RANK.AVG(B10,B$8:B$23,1)</f>
-        <v>12</v>
+        <f t="shared" ref="E10:F10" si="1">_xlfn.RANK.AVG(B10,B$9:B$24,1)</f>
+        <v>5.5</v>
       </c>
       <c r="F10" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
+      <c r="H10" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="I10" s="29">
+        <f>CORREL(E9:E24,F9:F24)</f>
+        <v>-0.74588967113847993</v>
+      </c>
       <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
       <c r="N10" s="11"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B11" s="11">
-        <v>5</v>
+        <v>6.1</v>
       </c>
       <c r="C11" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="11">
-        <f t="shared" ref="E11:F11" si="3">_xlfn.RANK.AVG(B11,B$8:B$23,1)</f>
-        <v>10</v>
+        <f t="shared" ref="E11:F11" si="2">_xlfn.RANK.AVG(B11,B$9:B$24,1)</f>
+        <v>12</v>
       </c>
       <c r="F11" s="11">
-        <f t="shared" si="3"/>
-        <v>4.5</v>
+        <f t="shared" si="2"/>
+        <v>9</v>
       </c>
       <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
       <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
       <c r="N11" s="11"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B12" s="11">
-        <v>4.2</v>
+        <v>5</v>
       </c>
       <c r="C12" s="11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="11">
-        <f t="shared" ref="E12:F12" si="4">_xlfn.RANK.AVG(B12,B$8:B$23,1)</f>
-        <v>8</v>
+        <f t="shared" ref="E12:F12" si="3">_xlfn.RANK.AVG(B12,B$9:B$24,1)</f>
+        <v>10</v>
       </c>
       <c r="F12" s="11">
-        <f t="shared" si="4"/>
-        <v>9</v>
+        <f t="shared" si="3"/>
+        <v>4.5</v>
       </c>
       <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
       <c r="J12" s="11"/>
       <c r="K12" s="11"/>
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
       <c r="N12" s="11"/>
     </row>
-    <row r="13" spans="1:14" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B13" s="11">
-        <v>2.5</v>
+        <v>4.2</v>
       </c>
       <c r="C13" s="11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="11">
-        <f t="shared" ref="E13:F13" si="5">_xlfn.RANK.AVG(B13,B$8:B$23,1)</f>
+        <f t="shared" ref="E13:F13" si="4">_xlfn.RANK.AVG(B13,B$9:B$24,1)</f>
+        <v>8</v>
+      </c>
+      <c r="F13" s="11">
+        <f t="shared" si="4"/>
+        <v>9</v>
+      </c>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="11"/>
+    </row>
+    <row r="14" spans="1:14" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="11">
+        <v>2.5</v>
+      </c>
+      <c r="C14" s="11">
+        <v>5</v>
+      </c>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11">
+        <f t="shared" ref="E14:F14" si="5">_xlfn.RANK.AVG(B14,B$9:B$24,1)</f>
         <v>1</v>
       </c>
-      <c r="F13" s="11">
+      <c r="F14" s="11">
         <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="G13" s="11"/>
-      <c r="H13" s="57" t="s">
-        <v>82</v>
-      </c>
-      <c r="I13" s="57"/>
-      <c r="J13" s="57"/>
-      <c r="K13" s="57"/>
-      <c r="L13" s="57"/>
-      <c r="M13" s="57"/>
-      <c r="N13" s="57"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B14" s="11">
+      <c r="G14" s="11"/>
+      <c r="H14" s="56" t="s">
+        <v>78</v>
+      </c>
+      <c r="I14" s="56"/>
+      <c r="J14" s="56"/>
+      <c r="K14" s="56"/>
+      <c r="L14" s="56"/>
+      <c r="M14" s="56"/>
+      <c r="N14" s="56"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B15" s="11">
         <v>3.2</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C15" s="11">
         <v>4</v>
       </c>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11">
-        <f t="shared" ref="E14:F14" si="6">_xlfn.RANK.AVG(B14,B$8:B$23,1)</f>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11">
+        <f t="shared" ref="E15:F15" si="6">_xlfn.RANK.AVG(B15,B$9:B$24,1)</f>
         <v>4</v>
       </c>
-      <c r="F14" s="11">
+      <c r="F15" s="11">
         <f t="shared" si="6"/>
         <v>14</v>
       </c>
-      <c r="G14" s="11"/>
-      <c r="H14" s="57"/>
-      <c r="I14" s="57"/>
-      <c r="J14" s="57"/>
-      <c r="K14" s="57"/>
-      <c r="L14" s="57"/>
-      <c r="M14" s="57"/>
-      <c r="N14" s="57"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="11">
+      <c r="G15" s="11"/>
+      <c r="H15" s="56"/>
+      <c r="I15" s="56"/>
+      <c r="J15" s="56"/>
+      <c r="K15" s="56"/>
+      <c r="L15" s="56"/>
+      <c r="M15" s="56"/>
+      <c r="N15" s="56"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B16" s="11">
         <v>6.8</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C16" s="11">
         <v>1</v>
       </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11">
-        <f t="shared" ref="E15:F15" si="7">_xlfn.RANK.AVG(B15,B$8:B$23,1)</f>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11">
+        <f t="shared" ref="E16:F16" si="7">_xlfn.RANK.AVG(B16,B$9:B$24,1)</f>
         <v>14</v>
       </c>
-      <c r="F15" s="11">
+      <c r="F16" s="11">
         <f t="shared" si="7"/>
         <v>2</v>
       </c>
-      <c r="G15" s="11"/>
-      <c r="H15" s="57"/>
-      <c r="I15" s="57"/>
-      <c r="J15" s="57"/>
-      <c r="K15" s="57"/>
-      <c r="L15" s="57"/>
-      <c r="M15" s="57"/>
-      <c r="N15" s="57"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="11">
+      <c r="G16" s="11"/>
+      <c r="H16" s="56"/>
+      <c r="I16" s="56"/>
+      <c r="J16" s="56"/>
+      <c r="K16" s="56"/>
+      <c r="L16" s="56"/>
+      <c r="M16" s="56"/>
+      <c r="N16" s="56"/>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B17" s="11">
         <v>8.1</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C17" s="11">
         <v>1</v>
       </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11">
-        <f t="shared" ref="E16:F16" si="8">_xlfn.RANK.AVG(B16,B$8:B$23,1)</f>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11">
+        <f t="shared" ref="E17:F17" si="8">_xlfn.RANK.AVG(B17,B$9:B$24,1)</f>
         <v>16</v>
       </c>
-      <c r="F16" s="11">
+      <c r="F17" s="11">
         <f t="shared" si="8"/>
         <v>2</v>
       </c>
-      <c r="G16" s="11"/>
-      <c r="H16" s="30"/>
-    </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B17" s="11">
+      <c r="G17" s="11"/>
+      <c r="H17" s="30"/>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B18" s="11">
         <v>2.8</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C18" s="11">
         <v>3</v>
       </c>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11">
-        <f t="shared" ref="E17:F17" si="9">_xlfn.RANK.AVG(B17,B$8:B$23,1)</f>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11">
+        <f t="shared" ref="E18:F18" si="9">_xlfn.RANK.AVG(B18,B$9:B$24,1)</f>
         <v>2</v>
       </c>
-      <c r="F17" s="11">
+      <c r="F18" s="11">
         <f t="shared" si="9"/>
         <v>9</v>
       </c>
-      <c r="G17" s="11"/>
-    </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B18" s="11">
+      <c r="G18" s="11"/>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B19" s="11">
         <v>3.4</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C19" s="11">
         <v>4</v>
       </c>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11">
-        <f t="shared" ref="E18:F18" si="10">_xlfn.RANK.AVG(B18,B$8:B$23,1)</f>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11">
+        <f t="shared" ref="E19:F19" si="10">_xlfn.RANK.AVG(B19,B$9:B$24,1)</f>
         <v>5.5</v>
       </c>
-      <c r="F18" s="11">
+      <c r="F19" s="11">
         <f t="shared" si="10"/>
         <v>14</v>
       </c>
-      <c r="G18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-    </row>
-    <row r="19" spans="2:14" ht="13" x14ac:dyDescent="0.3">
-      <c r="B19" s="11">
-        <v>6.3</v>
-      </c>
-      <c r="C19" s="11">
-        <v>2</v>
-      </c>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11">
-        <f t="shared" ref="E19:F19" si="11">_xlfn.RANK.AVG(B19,B$8:B$23,1)</f>
-        <v>13</v>
-      </c>
-      <c r="F19" s="11">
-        <f t="shared" si="11"/>
-        <v>4.5</v>
-      </c>
       <c r="G19" s="11"/>
-      <c r="H19" s="31" t="s">
-        <v>59</v>
-      </c>
-      <c r="I19" s="29">
-        <f>ABS(I9)*SQRT(COUNT(C8:C23)-2)/SQRT(1-I9^2)</f>
-        <v>4.1900485398298146</v>
-      </c>
       <c r="J19" s="11"/>
       <c r="K19" s="11"/>
       <c r="L19" s="11"/>
@@ -6968,27 +7091,27 @@
     </row>
     <row r="20" spans="2:14" ht="13" x14ac:dyDescent="0.3">
       <c r="B20" s="11">
-        <v>4.0999999999999996</v>
+        <v>6.3</v>
       </c>
       <c r="C20" s="11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D20" s="11"/>
       <c r="E20" s="11">
-        <f t="shared" ref="E20:F20" si="12">_xlfn.RANK.AVG(B20,B$8:B$23,1)</f>
-        <v>7</v>
+        <f t="shared" ref="E20:F20" si="11">_xlfn.RANK.AVG(B20,B$9:B$24,1)</f>
+        <v>13</v>
       </c>
       <c r="F20" s="11">
-        <f t="shared" si="12"/>
-        <v>9</v>
+        <f t="shared" si="11"/>
+        <v>4.5</v>
       </c>
       <c r="G20" s="11"/>
       <c r="H20" s="31" t="s">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="I20" s="29">
-        <f>TDIST(I19,SUM(C8:C23-2),2)</f>
-        <v>0.14914617078748418</v>
+        <f>ABS(I10)*SQRT(COUNT(C9:C24)-2)/SQRT(1-I10^2)</f>
+        <v>4.1900485398298146</v>
       </c>
       <c r="J20" s="11"/>
       <c r="K20" s="11"/>
@@ -6996,43 +7119,50 @@
       <c r="M20" s="11"/>
       <c r="N20" s="11"/>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" ht="13" x14ac:dyDescent="0.3">
       <c r="B21" s="11">
-        <v>3.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="C21" s="11">
         <v>3</v>
       </c>
       <c r="D21" s="11"/>
       <c r="E21" s="11">
-        <f t="shared" ref="E21:F21" si="13">_xlfn.RANK.AVG(B21,B$8:B$23,1)</f>
-        <v>3</v>
+        <f t="shared" ref="E21:F21" si="12">_xlfn.RANK.AVG(B21,B$9:B$24,1)</f>
+        <v>7</v>
       </c>
       <c r="F21" s="11">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>9</v>
       </c>
       <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
+      <c r="H21" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="I21" s="29">
+        <f>TDIST(I20,SUM(C9:C24-2),2)</f>
+        <v>0.14914617078748418</v>
+      </c>
       <c r="J21" s="11"/>
       <c r="K21" s="11"/>
       <c r="L21" s="11"/>
+      <c r="M21" s="11"/>
+      <c r="N21" s="11"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B22" s="11">
-        <v>4.9000000000000004</v>
+        <v>3.1</v>
       </c>
       <c r="C22" s="11">
         <v>3</v>
       </c>
       <c r="D22" s="11"/>
       <c r="E22" s="11">
-        <f t="shared" ref="E22:F22" si="14">_xlfn.RANK.AVG(B22,B$8:B$23,1)</f>
-        <v>9</v>
+        <f t="shared" ref="E22:F22" si="13">_xlfn.RANK.AVG(B22,B$9:B$24,1)</f>
+        <v>3</v>
       </c>
       <c r="F22" s="11">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>9</v>
       </c>
       <c r="G22" s="11"/>
@@ -7044,19 +7174,19 @@
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B23" s="11">
-        <v>7.2</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="C23" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D23" s="11"/>
       <c r="E23" s="11">
-        <f t="shared" ref="E23:F23" si="15">_xlfn.RANK.AVG(B23,B$8:B$23,1)</f>
-        <v>15</v>
+        <f t="shared" ref="E23:F23" si="14">_xlfn.RANK.AVG(B23,B$9:B$24,1)</f>
+        <v>9</v>
       </c>
       <c r="F23" s="11">
-        <f t="shared" si="15"/>
-        <v>2</v>
+        <f t="shared" si="14"/>
+        <v>9</v>
       </c>
       <c r="G23" s="11"/>
       <c r="H23" s="11"/>
@@ -7065,50 +7195,74 @@
       <c r="K23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="C25" s="11" t="s">
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B24" s="11">
+        <v>7.2</v>
+      </c>
+      <c r="C24" s="11">
+        <v>1</v>
+      </c>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11">
+        <f t="shared" ref="E24:F24" si="15">_xlfn.RANK.AVG(B24,B$9:B$24,1)</f>
+        <v>15</v>
+      </c>
+      <c r="F24" s="11">
+        <f t="shared" si="15"/>
+        <v>2</v>
+      </c>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="11"/>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C26" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G25" s="33"/>
-      <c r="H25" s="51"/>
-    </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="C26" s="28" t="s">
-        <v>22</v>
-      </c>
       <c r="G26" s="33"/>
-      <c r="H26" s="51"/>
+      <c r="H26" s="50"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C27" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="G27" s="20"/>
-      <c r="H27" s="51"/>
+        <v>22</v>
+      </c>
+      <c r="G27" s="33"/>
+      <c r="H27" s="50"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C28" s="28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G28" s="20"/>
-      <c r="H28" s="51"/>
+      <c r="H28" s="50"/>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C29" s="28" t="s">
-        <v>25</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="G29" s="20"/>
+      <c r="H29" s="50"/>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C30" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C31" s="28" t="s">
         <v>26</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="H13:N15"/>
+    <mergeCell ref="H14:N16"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -7135,7 +7289,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="13" x14ac:dyDescent="0.3">
@@ -7143,7 +7297,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:25" ht="13" x14ac:dyDescent="0.3">
@@ -7580,11 +7734,11 @@
       <c r="A20" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="38">
+      <c r="B20" s="37">
         <f>AVERAGE(B7:B18)</f>
         <v>4.2249999999999996</v>
       </c>
-      <c r="C20" s="38">
+      <c r="C20" s="37">
         <f>AVERAGE(C7:C18)</f>
         <v>5.1416666666666666</v>
       </c>
@@ -7613,7 +7767,7 @@
     </row>
     <row r="21" spans="1:25" ht="13" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="B21" s="29">
         <f>_xlfn.STDEV.S(B7:B18)</f>
@@ -7675,16 +7829,16 @@
     </row>
     <row r="23" spans="1:25" ht="39" x14ac:dyDescent="0.3">
       <c r="A23" s="11"/>
-      <c r="B23" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C23" s="44">
+      <c r="B23" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="43">
         <f>_xlfn.T.TEST(B7:B18,C7:C18,2,2)</f>
         <v>2.503154885551319E-3</v>
       </c>
       <c r="D23" s="11"/>
-      <c r="E23" s="45" t="s">
-        <v>86</v>
+      <c r="E23" s="44" t="s">
+        <v>81</v>
       </c>
       <c r="F23" s="11"/>
       <c r="G23" s="11"/>
@@ -7774,7 +7928,7 @@
   <dimension ref="A1:Y15"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.54296875" style="12" customWidth="1"/>
+    <col min="1" max="1" width="15.90625" style="12" customWidth="1"/>
     <col min="2" max="2" width="16.6328125" style="12" customWidth="1"/>
     <col min="3" max="4" width="25.26953125" style="12" customWidth="1"/>
     <col min="5" max="5" width="4.81640625" style="12" customWidth="1"/>
@@ -7784,12 +7938,12 @@
   <sheetData>
     <row r="1" spans="1:25" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="13" x14ac:dyDescent="0.3">
@@ -7797,7 +7951,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:25" ht="13" x14ac:dyDescent="0.3">
@@ -7805,10 +7959,10 @@
       <c r="B6" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="59" t="s">
+      <c r="C6" s="58" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="60"/>
+      <c r="D6" s="59"/>
       <c r="E6" s="11"/>
       <c r="F6" s="11"/>
       <c r="G6" s="11"/>
@@ -7936,7 +8090,7 @@
     </row>
     <row r="11" spans="1:25" ht="13" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
-        <v>45</v>
+        <v>118</v>
       </c>
       <c r="B11" s="31">
         <f t="shared" ref="B11:D11" si="0">SUM(B8:B9)</f>
@@ -7946,7 +8100,7 @@
         <f t="shared" si="0"/>
         <v>2520</v>
       </c>
-      <c r="D11" s="39">
+      <c r="D11" s="38">
         <f t="shared" si="0"/>
         <v>2520</v>
       </c>
@@ -8002,16 +8156,16 @@
     <row r="13" spans="1:25" ht="39" x14ac:dyDescent="0.3">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
-      <c r="C13" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" s="46">
+      <c r="C13" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="D13" s="45">
         <f>CHITEST(C8:C9,D8:D9)</f>
         <v>2.2006076735235521E-2</v>
       </c>
       <c r="E13" s="11"/>
-      <c r="F13" s="45" t="s">
-        <v>87</v>
+      <c r="F13" s="44" t="s">
+        <v>82</v>
       </c>
       <c r="G13" s="11"/>
       <c r="H13" s="11"/>
@@ -8034,9 +8188,9 @@
       <c r="Y13" s="11"/>
     </row>
     <row r="15" spans="1:25" ht="39" x14ac:dyDescent="0.3">
-      <c r="D15" s="47"/>
-      <c r="F15" s="48" t="s">
-        <v>88</v>
+      <c r="D15" s="46"/>
+      <c r="F15" s="47" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -8067,12 +8221,12 @@
   <sheetData>
     <row r="1" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="13" x14ac:dyDescent="0.3">
@@ -8080,7 +8234,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="13" x14ac:dyDescent="0.3">
@@ -8110,11 +8264,11 @@
       <c r="E7" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="40">
+      <c r="F7" s="39">
         <f t="shared" ref="F7:G7" si="0">AVERAGE(B7:B18)</f>
         <v>4.2249999999999996</v>
       </c>
-      <c r="G7" s="40">
+      <c r="G7" s="39">
         <f t="shared" si="0"/>
         <v>5.1416666666666666</v>
       </c>
@@ -8130,13 +8284,13 @@
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="F8" s="40">
+        <v>94</v>
+      </c>
+      <c r="F8" s="39">
         <f>_xlfn.STDEV.S(B7:B18)</f>
         <v>0.65799281565572354</v>
       </c>
-      <c r="G8" s="40">
+      <c r="G8" s="39">
         <f>_xlfn.STDEV.S(C7:C18)</f>
         <v>0.65845319200426822</v>
       </c>
@@ -8152,7 +8306,7 @@
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="25" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="F9" s="11">
         <f>COUNT(B7:B18)</f>
@@ -8163,7 +8317,7 @@
         <v>12</v>
       </c>
       <c r="H9" s="11"/>
-      <c r="L9" s="50">
+      <c r="L9" s="49">
         <v>0.95</v>
       </c>
     </row>
@@ -8176,7 +8330,7 @@
         <v>4.7</v>
       </c>
       <c r="E10" s="5"/>
-      <c r="L10" s="50">
+      <c r="L10" s="49">
         <v>0.97499999999999998</v>
       </c>
     </row>
@@ -8190,13 +8344,13 @@
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="25" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="F11" s="21">
         <v>0.95</v>
       </c>
       <c r="H11" s="11"/>
-      <c r="L11" s="50">
+      <c r="L11" s="49">
         <v>0.99</v>
       </c>
     </row>
@@ -8210,7 +8364,7 @@
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="25" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="F12" s="21">
         <f>1-F11</f>
@@ -8218,7 +8372,7 @@
       </c>
       <c r="G12" s="11"/>
       <c r="H12" s="11"/>
-      <c r="L12" s="50">
+      <c r="L12" s="49">
         <v>0.999</v>
       </c>
     </row>
@@ -8243,13 +8397,13 @@
       </c>
       <c r="D14" s="11"/>
       <c r="E14" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="F14" s="40">
+        <v>97</v>
+      </c>
+      <c r="F14" s="39">
         <f>_xlfn.CONFIDENCE.T(F12,F8,F9)</f>
         <v>0.41806868954898424</v>
       </c>
-      <c r="G14" s="40">
+      <c r="G14" s="39">
         <f>_xlfn.CONFIDENCE.T(F12,G8,G9)</f>
         <v>0.41836119872561345</v>
       </c>
@@ -8265,13 +8419,13 @@
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="F15" s="41" t="str">
+        <v>98</v>
+      </c>
+      <c r="F15" s="40" t="str">
         <f>ROUND(F7,2) &amp;" +/- " &amp; ROUND(F14,2)</f>
         <v>4,23 +/- 0,42</v>
       </c>
-      <c r="G15" s="41" t="str">
+      <c r="G15" s="40" t="str">
         <f>ROUND(G7,2) &amp;" +/- " &amp; ROUND(G14,2)</f>
         <v>5,14 +/- 0,42</v>
       </c>
@@ -8321,11 +8475,11 @@
       <c r="E18" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="F18" s="41">
+      <c r="F18" s="40">
         <f>F19-F14</f>
         <v>3.8069313104510156</v>
       </c>
-      <c r="G18" s="41">
+      <c r="G18" s="40">
         <f>G19-G14</f>
         <v>4.7233054679410529</v>
       </c>
@@ -8339,11 +8493,11 @@
       <c r="E19" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="F19" s="41">
+      <c r="F19" s="40">
         <f>F7</f>
         <v>4.2249999999999996</v>
       </c>
-      <c r="G19" s="41">
+      <c r="G19" s="40">
         <f>G7</f>
         <v>5.1416666666666666</v>
       </c>
@@ -8357,19 +8511,19 @@
       <c r="E20" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="F20" s="41">
+      <c r="F20" s="40">
         <f>F19+F14</f>
         <v>4.6430686895489837</v>
       </c>
-      <c r="G20" s="41">
+      <c r="G20" s="40">
         <f>G19+G14</f>
         <v>5.5600278653922803</v>
       </c>
       <c r="H20" s="11"/>
     </row>
     <row r="21" spans="1:23" ht="13" x14ac:dyDescent="0.3">
-      <c r="A21" s="21" t="s">
-        <v>67</v>
+      <c r="A21" s="25" t="s">
+        <v>80</v>
       </c>
       <c r="B21" s="29">
         <f>_xlfn.T.TEST(B7:B18,C7:C18,2,2)</f>
@@ -8389,11 +8543,11 @@
         <f>"Do intervals overlap?" &amp; IF(F22&lt;G22," No!"," Yes!")</f>
         <v>Do intervals overlap? No!</v>
       </c>
-      <c r="F22" s="41">
+      <c r="F22" s="40">
         <f>MIN(F20,G20)</f>
         <v>4.6430686895489837</v>
       </c>
-      <c r="G22" s="41">
+      <c r="G22" s="40">
         <f>MAX(F18,G18)</f>
         <v>4.7233054679410529</v>
       </c>
@@ -8416,8 +8570,8 @@
     </row>
     <row r="23" spans="1:23" ht="91" x14ac:dyDescent="0.3">
       <c r="D23" s="11"/>
-      <c r="E23" s="49" t="s">
-        <v>98</v>
+      <c r="E23" s="48" t="s">
+        <v>120</v>
       </c>
       <c r="F23" s="11"/>
       <c r="G23" s="11"/>

</xml_diff>